<commit_message>
vault backup: 2026-07-03 16:21:46
</commit_message>
<xml_diff>
--- a/Daily-Task-List/Knowledge_Base/WTO-IOTC/教学大纲/《国际渔业法》/相关书籍/书籍链接.xlsx
+++ b/Daily-Task-List/Knowledge_Base/WTO-IOTC/教学大纲/《国际渔业法》/相关书籍/书籍链接.xlsx
@@ -1,13 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\1_Learning_Record\1_Typora\My-NoteBook\Daily-Task-List\Knowledge_Base\WTO-IOTC\教学大纲\《国际渔业法》\相关书籍\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{661F47E9-4627-4548-AE12-DA060D876ABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="参考教材与阅读书目" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -18,12 +24,106 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="17">
+  <si>
+    <t>书籍</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>是否可下载</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>链接</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>✔</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.gbv.de/dms/spk/sbb/toc/277908760.pdf</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://api.pageplace.de/preview/DT0400.9781009035910_A47731355/preview-9781009035910_A47731355.pdf</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://openknowledge.fao.org/server/api/core/bitstreams/23312a48-cb99-4abf-b7e9-4f2f38604695/content</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>类别</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>参考教材</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>阅读书目</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Code Of Conduct For Responsible Fisheries</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>The International Law of the Sea</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>The New International Law of Fisheries</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://openknowledge.fao.org/server/api/core/bitstreams/515b81dc-ad65-41c9-ab02-6ff081103cc3/content</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Agreement on Port State Measures to Prevent, Deter and Eliminate Illegal, Unreported and Unregulated Fishing (PSMA)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.wto.org/english/tratop_e/rulesneg_e/fish_e/agreement_on_fisheries_subsidies_information_session_22_may_2025_final.pdf</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>THE WTO AGREEMENT ON FISHERIES SUBSIDIES</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="等线"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI Symbol"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -46,14 +146,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  <cellStyles count="2">
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="超链接" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -330,10 +434,109 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="102.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="102.5" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="102.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{7065177A-F66B-4FC1-9BB0-215465FF10E4}"/>
+    <hyperlink ref="D3" r:id="rId2" xr:uid="{A974B0D1-53B1-4245-A623-8135AC57E345}"/>
+    <hyperlink ref="D4" r:id="rId3" xr:uid="{8581CF74-BF57-4587-804A-6DF07BC4062E}"/>
+    <hyperlink ref="D5" r:id="rId4" xr:uid="{DEF82C2E-8F9F-4EBA-9084-452EC88D4C9E}"/>
+    <hyperlink ref="D6" r:id="rId5" xr:uid="{D0418401-7BDD-4F85-9E6C-6EF4716DE911}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-07-03 16:43:59
</commit_message>
<xml_diff>
--- a/Daily-Task-List/Knowledge_Base/WTO-IOTC/教学大纲/《国际渔业法》/相关书籍/书籍链接.xlsx
+++ b/Daily-Task-List/Knowledge_Base/WTO-IOTC/教学大纲/《国际渔业法》/相关书籍/书籍链接.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\1_Learning_Record\1_Typora\My-NoteBook\Daily-Task-List\Knowledge_Base\WTO-IOTC\教学大纲\《国际渔业法》\相关书籍\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{661F47E9-4627-4548-AE12-DA060D876ABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7BA2EC6-27C3-4303-9338-37CB0239D8FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="20">
   <si>
     <t>书籍</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -92,6 +92,18 @@
   </si>
   <si>
     <t>THE WTO AGREEMENT ON FISHERIES SUBSIDIES</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.iisd.org/system/files/2023-03/wto-agreement-fisheries-subsidies-readers-guide.pdf</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>WTO读者指南</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>The WTO Agreement on Fisheries Subsidies: A Reader’s Guide</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -99,7 +111,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -128,13 +140,34 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="2"/>
+      <name val="等线"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="2"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -150,10 +183,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -435,7 +470,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="102.5" bestFit="1" customWidth="1"/>
@@ -445,16 +480,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
     </row>
@@ -526,6 +561,20 @@
       </c>
       <c r="D6" s="2" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -536,6 +585,7 @@
     <hyperlink ref="D4" r:id="rId3" xr:uid="{8581CF74-BF57-4587-804A-6DF07BC4062E}"/>
     <hyperlink ref="D5" r:id="rId4" xr:uid="{DEF82C2E-8F9F-4EBA-9084-452EC88D4C9E}"/>
     <hyperlink ref="D6" r:id="rId5" xr:uid="{D0418401-7BDD-4F85-9E6C-6EF4716DE911}"/>
+    <hyperlink ref="D7" r:id="rId6" xr:uid="{67ADFC54-6F2C-4FD0-B417-140F6044E390}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
vault backup: 2026-07-03 16:50:25
</commit_message>
<xml_diff>
--- a/Daily-Task-List/Knowledge_Base/WTO-IOTC/教学大纲/《国际渔业法》/相关书籍/书籍链接.xlsx
+++ b/Daily-Task-List/Knowledge_Base/WTO-IOTC/教学大纲/《国际渔业法》/相关书籍/书籍链接.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\1_Learning_Record\1_Typora\My-NoteBook\Daily-Task-List\Knowledge_Base\WTO-IOTC\教学大纲\《国际渔业法》\相关书籍\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7BA2EC6-27C3-4303-9338-37CB0239D8FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AA74925-4267-4273-B111-EB846E01B8E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="23">
   <si>
     <t>书籍</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -104,6 +104,18 @@
   </si>
   <si>
     <t>The WTO Agreement on Fisheries Subsidies: A Reader’s Guide</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>❌</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>《国际渔业》（海洋渔业类专业用·面向21世纪课程教材） 中国农业出版社。ISBN：7109068625</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>华敬炘：《渔业法学通论》（上下册） 中国海洋大学出版社，2017。ISBN（下册）：978-7-5670-1448-0</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -470,7 +482,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="102.5" bestFit="1" customWidth="1"/>
@@ -575,6 +587,28 @@
       </c>
       <c r="D7" s="2" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>